<commit_message>
Update published PMQ dashboard workbook
</commit_message>
<xml_diff>
--- a/test/published_reports/pmq_client_dashboard.xlsx
+++ b/test/published_reports/pmq_client_dashboard.xlsx
@@ -1618,7 +1618,7 @@
     <row r="31">
       <c r="A31" s="22" t="inlineStr">
         <is>
-          <t>Average overall performance score is 85.9, which is currently stable.</t>
+          <t>Average overall performance score is 85.8, which is currently stable.</t>
         </is>
       </c>
       <c r="B31" s="23" t="n"/>
@@ -2413,7 +2413,7 @@
         </is>
       </c>
       <c r="B9" s="31" t="n">
-        <v>89</v>
+        <v>88.8</v>
       </c>
     </row>
     <row r="10">
@@ -2443,7 +2443,7 @@
         </is>
       </c>
       <c r="B12" s="31" t="n">
-        <v>75</v>
+        <v>75.59999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="B13" s="31" t="n">
-        <v>85.3</v>
+        <v>85.2</v>
       </c>
     </row>
     <row r="14">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="B14" s="31" t="n">
-        <v>85.90000000000001</v>
+        <v>85.8</v>
       </c>
     </row>
   </sheetData>
@@ -2790,7 +2790,7 @@
     <row r="5">
       <c r="A5" s="31" t="inlineStr">
         <is>
-          <t>Average overall performance score is 85.9, which is currently stable.</t>
+          <t>Average overall performance score is 85.8, which is currently stable.</t>
         </is>
       </c>
       <c r="B5" s="31" t="inlineStr">
@@ -3027,22 +3027,22 @@
         </is>
       </c>
       <c r="G2" s="31" t="n">
-        <v>86</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="H2" s="31" t="n">
-        <v>86.09999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="I2" s="31" t="n">
-        <v>89.8</v>
+        <v>90</v>
       </c>
       <c r="J2" s="31" t="n">
         <v>80.5</v>
       </c>
       <c r="K2" s="31" t="n">
-        <v>98</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="L2" s="31" t="n">
-        <v>64.2</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3">
@@ -3077,22 +3077,22 @@
         </is>
       </c>
       <c r="G3" s="31" t="n">
-        <v>85.7</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="H3" s="31" t="n">
-        <v>85.8</v>
+        <v>86.2</v>
       </c>
       <c r="I3" s="31" t="n">
-        <v>89</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="J3" s="31" t="n">
         <v>81</v>
       </c>
       <c r="K3" s="31" t="n">
-        <v>92.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="L3" s="31" t="n">
-        <v>74.2</v>
+        <v>76.2</v>
       </c>
     </row>
     <row r="4">
@@ -3127,13 +3127,13 @@
         </is>
       </c>
       <c r="G4" s="31" t="n">
-        <v>83.2</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H4" s="31" t="n">
-        <v>84.40000000000001</v>
+        <v>84.7</v>
       </c>
       <c r="I4" s="31" t="n">
-        <v>89.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="J4" s="31" t="n">
         <v>74.5</v>
@@ -3142,7 +3142,7 @@
         <v>99</v>
       </c>
       <c r="L4" s="31" t="n">
-        <v>75.8</v>
+        <v>77.59999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -3177,19 +3177,19 @@
         </is>
       </c>
       <c r="G5" s="31" t="n">
-        <v>86.3</v>
+        <v>86.2</v>
       </c>
       <c r="H5" s="31" t="n">
         <v>86.7</v>
       </c>
       <c r="I5" s="31" t="n">
-        <v>90</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="J5" s="31" t="n">
         <v>81</v>
       </c>
       <c r="K5" s="31" t="n">
-        <v>94.90000000000001</v>
+        <v>95.2</v>
       </c>
       <c r="L5" s="31" t="n">
         <v>77.59999999999999</v>
@@ -3227,13 +3227,13 @@
         </is>
       </c>
       <c r="G6" s="31" t="n">
-        <v>86.09999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="H6" s="31" t="n">
-        <v>87.2</v>
+        <v>87.3</v>
       </c>
       <c r="I6" s="31" t="n">
-        <v>89.7</v>
+        <v>89.8</v>
       </c>
       <c r="J6" s="31" t="n">
         <v>81</v>
@@ -3277,22 +3277,22 @@
         </is>
       </c>
       <c r="G7" s="31" t="n">
-        <v>86</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="H7" s="31" t="n">
-        <v>86</v>
+        <v>86.2</v>
       </c>
       <c r="I7" s="31" t="n">
-        <v>90.59999999999999</v>
+        <v>90.7</v>
       </c>
       <c r="J7" s="31" t="n">
         <v>79.5</v>
       </c>
       <c r="K7" s="31" t="n">
-        <v>92.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="L7" s="31" t="n">
-        <v>72.40000000000001</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -3327,22 +3327,22 @@
         </is>
       </c>
       <c r="G8" s="31" t="n">
-        <v>86.5</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="H8" s="31" t="n">
-        <v>86.59999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="I8" s="31" t="n">
-        <v>90.7</v>
+        <v>90.8</v>
       </c>
       <c r="J8" s="31" t="n">
         <v>80.5</v>
       </c>
       <c r="K8" s="31" t="n">
-        <v>93.90000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="L8" s="31" t="n">
-        <v>73.40000000000001</v>
+        <v>73.8</v>
       </c>
     </row>
     <row r="9">
@@ -3380,19 +3380,19 @@
         <v>85.09999999999999</v>
       </c>
       <c r="H9" s="31" t="n">
-        <v>85.2</v>
+        <v>85.3</v>
       </c>
       <c r="I9" s="31" t="n">
-        <v>89</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="J9" s="31" t="n">
         <v>79.5</v>
       </c>
       <c r="K9" s="31" t="n">
-        <v>94.90000000000001</v>
+        <v>95.2</v>
       </c>
       <c r="L9" s="31" t="n">
-        <v>67.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -3427,13 +3427,13 @@
         </is>
       </c>
       <c r="G10" s="31" t="n">
-        <v>86.2</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="H10" s="31" t="n">
-        <v>87.09999999999999</v>
+        <v>87.3</v>
       </c>
       <c r="I10" s="31" t="n">
-        <v>89.90000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="J10" s="31" t="n">
         <v>81</v>
@@ -3442,7 +3442,7 @@
         <v>100</v>
       </c>
       <c r="L10" s="31" t="n">
-        <v>76.59999999999999</v>
+        <v>78.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -3477,22 +3477,22 @@
         </is>
       </c>
       <c r="G11" s="31" t="n">
-        <v>86.09999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="H11" s="31" t="n">
-        <v>87.3</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="I11" s="31" t="n">
-        <v>90.40000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="J11" s="31" t="n">
         <v>80</v>
       </c>
       <c r="K11" s="31" t="n">
-        <v>94.90000000000001</v>
+        <v>95.2</v>
       </c>
       <c r="L11" s="31" t="n">
-        <v>91.59999999999999</v>
+        <v>90.8</v>
       </c>
     </row>
     <row r="12">
@@ -3527,22 +3527,22 @@
         </is>
       </c>
       <c r="G12" s="31" t="n">
-        <v>86.5</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="H12" s="31" t="n">
         <v>86.5</v>
       </c>
       <c r="I12" s="31" t="n">
-        <v>90</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="J12" s="31" t="n">
         <v>81.5</v>
       </c>
       <c r="K12" s="31" t="n">
-        <v>97</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="L12" s="31" t="n">
-        <v>65.8</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13">
@@ -3577,22 +3577,22 @@
         </is>
       </c>
       <c r="G13" s="31" t="n">
-        <v>81.90000000000001</v>
+        <v>82.3</v>
       </c>
       <c r="H13" s="31" t="n">
-        <v>82.59999999999999</v>
+        <v>83</v>
       </c>
       <c r="I13" s="31" t="n">
-        <v>83.3</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="J13" s="31" t="n">
         <v>80</v>
       </c>
       <c r="K13" s="31" t="n">
-        <v>94.90000000000001</v>
+        <v>95.2</v>
       </c>
       <c r="L13" s="31" t="n">
-        <v>69.2</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14">
@@ -3627,22 +3627,22 @@
         </is>
       </c>
       <c r="G14" s="31" t="n">
-        <v>86.09999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="H14" s="31" t="n">
-        <v>87.2</v>
+        <v>82.3</v>
       </c>
       <c r="I14" s="31" t="n">
-        <v>90.3</v>
+        <v>82.2</v>
       </c>
       <c r="J14" s="31" t="n">
         <v>80</v>
       </c>
       <c r="K14" s="31" t="n">
-        <v>98</v>
+        <v>93.3</v>
       </c>
       <c r="L14" s="31" t="n">
-        <v>85</v>
+        <v>78.40000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -3677,22 +3677,22 @@
         </is>
       </c>
       <c r="G15" s="31" t="n">
-        <v>84.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="H15" s="31" t="n">
-        <v>84.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="I15" s="31" t="n">
-        <v>88.40000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="J15" s="31" t="n">
         <v>80</v>
       </c>
       <c r="K15" s="31" t="n">
-        <v>92.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="L15" s="31" t="n">
-        <v>67.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -3742,7 +3742,7 @@
         <v>100</v>
       </c>
       <c r="L16" s="31" t="n">
-        <v>86.59999999999999</v>
+        <v>86.19999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -3777,22 +3777,22 @@
         </is>
       </c>
       <c r="G17" s="31" t="n">
-        <v>83</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="H17" s="31" t="n">
-        <v>83</v>
+        <v>83.2</v>
       </c>
       <c r="I17" s="31" t="n">
-        <v>85.09999999999999</v>
+        <v>85.3</v>
       </c>
       <c r="J17" s="31" t="n">
         <v>80</v>
       </c>
       <c r="K17" s="31" t="n">
-        <v>90.90000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="L17" s="31" t="n">
-        <v>66.59999999999999</v>
+        <v>69.2</v>
       </c>
     </row>
     <row r="18">
@@ -3830,19 +3830,19 @@
         <v>86.3</v>
       </c>
       <c r="H18" s="31" t="n">
-        <v>87.3</v>
+        <v>87.5</v>
       </c>
       <c r="I18" s="31" t="n">
-        <v>90.3</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="J18" s="31" t="n">
         <v>80.5</v>
       </c>
       <c r="K18" s="31" t="n">
-        <v>98</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="L18" s="31" t="n">
-        <v>84.2</v>
+        <v>85.39999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -3877,22 +3877,22 @@
         </is>
       </c>
       <c r="G19" s="31" t="n">
-        <v>82.8</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="H19" s="31" t="n">
-        <v>83.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="I19" s="31" t="n">
-        <v>84.8</v>
+        <v>85</v>
       </c>
       <c r="J19" s="31" t="n">
         <v>80</v>
       </c>
       <c r="K19" s="31" t="n">
-        <v>97</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="L19" s="31" t="n">
-        <v>67.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -3942,7 +3942,7 @@
         <v>99</v>
       </c>
       <c r="L20" s="31" t="n">
-        <v>79.2</v>
+        <v>80.8</v>
       </c>
     </row>
     <row r="21">
@@ -3977,13 +3977,13 @@
         </is>
       </c>
       <c r="G21" s="31" t="n">
-        <v>85.5</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="H21" s="31" t="n">
-        <v>86.7</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="I21" s="31" t="n">
-        <v>89.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="J21" s="31" t="n">
         <v>80</v>
@@ -3992,7 +3992,7 @@
         <v>99</v>
       </c>
       <c r="L21" s="31" t="n">
-        <v>83.40000000000001</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22">
@@ -4027,22 +4027,22 @@
         </is>
       </c>
       <c r="G22" s="31" t="n">
-        <v>85.90000000000001</v>
+        <v>86</v>
       </c>
       <c r="H22" s="31" t="n">
-        <v>85.59999999999999</v>
+        <v>85.8</v>
       </c>
       <c r="I22" s="31" t="n">
-        <v>90</v>
+        <v>90.2</v>
       </c>
       <c r="J22" s="31" t="n">
         <v>80</v>
       </c>
       <c r="K22" s="31" t="n">
-        <v>93.90000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="L22" s="31" t="n">
-        <v>64.2</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -4251,7 +4251,7 @@
         </is>
       </c>
       <c r="H2" s="31" t="n">
-        <v>98</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="I2" s="31" t="inlineStr">
         <is>
@@ -4259,7 +4259,7 @@
         </is>
       </c>
       <c r="J2" s="31" t="n">
-        <v>64.2</v>
+        <v>67</v>
       </c>
       <c r="K2" s="31" t="inlineStr">
         <is>
@@ -4273,17 +4273,17 @@
         <v>9</v>
       </c>
       <c r="N2" s="31" t="n">
-        <v>97.40000000000001</v>
+        <v>97.8</v>
       </c>
       <c r="O2" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P2" s="31" t="n">
-        <v>89.8</v>
+        <v>90</v>
       </c>
       <c r="Q2" s="31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="R2" s="31" t="n">
@@ -4298,7 +4298,7 @@
         </is>
       </c>
       <c r="U2" s="31" t="n">
-        <v>86</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="V2" s="31" t="inlineStr">
         <is>
@@ -4306,7 +4306,7 @@
         </is>
       </c>
       <c r="W2" s="31" t="n">
-        <v>86.09999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="X2" s="31" t="inlineStr">
         <is>
@@ -4356,7 +4356,7 @@
         </is>
       </c>
       <c r="H3" s="31" t="n">
-        <v>92.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="I3" s="31" t="inlineStr">
         <is>
@@ -4364,7 +4364,7 @@
         </is>
       </c>
       <c r="J3" s="31" t="n">
-        <v>74.2</v>
+        <v>76.2</v>
       </c>
       <c r="K3" s="31" t="inlineStr">
         <is>
@@ -4378,13 +4378,13 @@
         <v>9</v>
       </c>
       <c r="N3" s="31" t="n">
-        <v>96.09999999999999</v>
+        <v>96.8</v>
       </c>
       <c r="O3" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P3" s="31" t="n">
-        <v>89</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="Q3" s="31" t="inlineStr">
         <is>
@@ -4403,7 +4403,7 @@
         </is>
       </c>
       <c r="U3" s="31" t="n">
-        <v>85.7</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="V3" s="31" t="inlineStr">
         <is>
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="W3" s="31" t="n">
-        <v>85.8</v>
+        <v>86.2</v>
       </c>
       <c r="X3" s="31" t="inlineStr">
         <is>
@@ -4469,7 +4469,7 @@
         </is>
       </c>
       <c r="J4" s="31" t="n">
-        <v>75.8</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="K4" s="31" t="inlineStr">
         <is>
@@ -4483,13 +4483,13 @@
         <v>9</v>
       </c>
       <c r="N4" s="31" t="n">
-        <v>97.5</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="O4" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P4" s="31" t="n">
-        <v>89.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="Q4" s="31" t="inlineStr">
         <is>
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="U4" s="31" t="n">
-        <v>83.2</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="V4" s="31" t="inlineStr">
         <is>
@@ -4516,7 +4516,7 @@
         </is>
       </c>
       <c r="W4" s="31" t="n">
-        <v>84.40000000000001</v>
+        <v>84.7</v>
       </c>
       <c r="X4" s="31" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         </is>
       </c>
       <c r="H5" s="31" t="n">
-        <v>94.90000000000001</v>
+        <v>95.2</v>
       </c>
       <c r="I5" s="31" t="inlineStr">
         <is>
@@ -4588,17 +4588,17 @@
         <v>9</v>
       </c>
       <c r="N5" s="31" t="n">
-        <v>97.2</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="O5" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P5" s="31" t="n">
-        <v>90</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="Q5" s="31" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="R5" s="31" t="n">
@@ -4613,7 +4613,7 @@
         </is>
       </c>
       <c r="U5" s="31" t="n">
-        <v>86.3</v>
+        <v>86.2</v>
       </c>
       <c r="V5" s="31" t="inlineStr">
         <is>
@@ -4693,13 +4693,13 @@
         <v>9</v>
       </c>
       <c r="N6" s="31" t="n">
-        <v>97.7</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="O6" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P6" s="31" t="n">
-        <v>89.7</v>
+        <v>89.8</v>
       </c>
       <c r="Q6" s="31" t="inlineStr">
         <is>
@@ -4718,7 +4718,7 @@
         </is>
       </c>
       <c r="U6" s="31" t="n">
-        <v>86.09999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="V6" s="31" t="inlineStr">
         <is>
@@ -4726,7 +4726,7 @@
         </is>
       </c>
       <c r="W6" s="31" t="n">
-        <v>87.2</v>
+        <v>87.3</v>
       </c>
       <c r="X6" s="31" t="inlineStr">
         <is>
@@ -4776,7 +4776,7 @@
         </is>
       </c>
       <c r="H7" s="31" t="n">
-        <v>92.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="I7" s="31" t="inlineStr">
         <is>
@@ -4784,7 +4784,7 @@
         </is>
       </c>
       <c r="J7" s="31" t="n">
-        <v>72.40000000000001</v>
+        <v>73</v>
       </c>
       <c r="K7" s="31" t="inlineStr">
         <is>
@@ -4798,13 +4798,13 @@
         <v>9</v>
       </c>
       <c r="N7" s="31" t="n">
-        <v>98.90000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="O7" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P7" s="31" t="n">
-        <v>90.59999999999999</v>
+        <v>90.7</v>
       </c>
       <c r="Q7" s="31" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
         </is>
       </c>
       <c r="U7" s="31" t="n">
-        <v>86</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="V7" s="31" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         </is>
       </c>
       <c r="W7" s="31" t="n">
-        <v>86</v>
+        <v>86.2</v>
       </c>
       <c r="X7" s="31" t="inlineStr">
         <is>
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="H8" s="31" t="n">
-        <v>93.90000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="I8" s="31" t="inlineStr">
         <is>
@@ -4889,7 +4889,7 @@
         </is>
       </c>
       <c r="J8" s="31" t="n">
-        <v>73.40000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="K8" s="31" t="inlineStr">
         <is>
@@ -4903,13 +4903,13 @@
         <v>9</v>
       </c>
       <c r="N8" s="31" t="n">
-        <v>99.09999999999999</v>
+        <v>99.3</v>
       </c>
       <c r="O8" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P8" s="31" t="n">
-        <v>90.7</v>
+        <v>90.8</v>
       </c>
       <c r="Q8" s="31" t="inlineStr">
         <is>
@@ -4928,7 +4928,7 @@
         </is>
       </c>
       <c r="U8" s="31" t="n">
-        <v>86.5</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="V8" s="31" t="inlineStr">
         <is>
@@ -4936,7 +4936,7 @@
         </is>
       </c>
       <c r="W8" s="31" t="n">
-        <v>86.59999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="X8" s="31" t="inlineStr">
         <is>
@@ -4986,7 +4986,7 @@
         </is>
       </c>
       <c r="H9" s="31" t="n">
-        <v>94.90000000000001</v>
+        <v>95.2</v>
       </c>
       <c r="I9" s="31" t="inlineStr">
         <is>
@@ -4994,7 +4994,7 @@
         </is>
       </c>
       <c r="J9" s="31" t="n">
-        <v>67.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="K9" s="31" t="inlineStr">
         <is>
@@ -5008,13 +5008,13 @@
         <v>9</v>
       </c>
       <c r="N9" s="31" t="n">
-        <v>95.5</v>
+        <v>95.7</v>
       </c>
       <c r="O9" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P9" s="31" t="n">
-        <v>89</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="Q9" s="31" t="inlineStr">
         <is>
@@ -5041,7 +5041,7 @@
         </is>
       </c>
       <c r="W9" s="31" t="n">
-        <v>85.2</v>
+        <v>85.3</v>
       </c>
       <c r="X9" s="31" t="inlineStr">
         <is>
@@ -5099,7 +5099,7 @@
         </is>
       </c>
       <c r="J10" s="31" t="n">
-        <v>76.59999999999999</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="K10" s="31" t="inlineStr">
         <is>
@@ -5113,17 +5113,17 @@
         <v>9</v>
       </c>
       <c r="N10" s="31" t="n">
-        <v>98.59999999999999</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="O10" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P10" s="31" t="n">
-        <v>89.90000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="Q10" s="31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="R10" s="31" t="n">
@@ -5138,7 +5138,7 @@
         </is>
       </c>
       <c r="U10" s="31" t="n">
-        <v>86.2</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="V10" s="31" t="inlineStr">
         <is>
@@ -5146,7 +5146,7 @@
         </is>
       </c>
       <c r="W10" s="31" t="n">
-        <v>87.09999999999999</v>
+        <v>87.3</v>
       </c>
       <c r="X10" s="31" t="inlineStr">
         <is>
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="H11" s="31" t="n">
-        <v>94.90000000000001</v>
+        <v>95.2</v>
       </c>
       <c r="I11" s="31" t="inlineStr">
         <is>
@@ -5204,7 +5204,7 @@
         </is>
       </c>
       <c r="J11" s="31" t="n">
-        <v>91.59999999999999</v>
+        <v>90.8</v>
       </c>
       <c r="K11" s="31" t="inlineStr">
         <is>
@@ -5218,13 +5218,13 @@
         <v>9</v>
       </c>
       <c r="N11" s="31" t="n">
-        <v>98</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="O11" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P11" s="31" t="n">
-        <v>90.40000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="Q11" s="31" t="inlineStr">
         <is>
@@ -5243,7 +5243,7 @@
         </is>
       </c>
       <c r="U11" s="31" t="n">
-        <v>86.09999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="V11" s="31" t="inlineStr">
         <is>
@@ -5251,7 +5251,7 @@
         </is>
       </c>
       <c r="W11" s="31" t="n">
-        <v>87.3</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="X11" s="31" t="inlineStr">
         <is>
@@ -5301,7 +5301,7 @@
         </is>
       </c>
       <c r="H12" s="31" t="n">
-        <v>97</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="I12" s="31" t="inlineStr">
         <is>
@@ -5309,7 +5309,7 @@
         </is>
       </c>
       <c r="J12" s="31" t="n">
-        <v>65.8</v>
+        <v>67</v>
       </c>
       <c r="K12" s="31" t="inlineStr">
         <is>
@@ -5323,17 +5323,17 @@
         <v>9</v>
       </c>
       <c r="N12" s="31" t="n">
-        <v>97.5</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="O12" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P12" s="31" t="n">
-        <v>90</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="Q12" s="31" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="R12" s="31" t="n">
@@ -5348,7 +5348,7 @@
         </is>
       </c>
       <c r="U12" s="31" t="n">
-        <v>86.5</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="V12" s="31" t="inlineStr">
         <is>
@@ -5406,7 +5406,7 @@
         </is>
       </c>
       <c r="H13" s="31" t="n">
-        <v>94.90000000000001</v>
+        <v>95.2</v>
       </c>
       <c r="I13" s="31" t="inlineStr">
         <is>
@@ -5414,11 +5414,11 @@
         </is>
       </c>
       <c r="J13" s="31" t="n">
-        <v>69.2</v>
+        <v>70</v>
       </c>
       <c r="K13" s="31" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L13" s="31" t="n">
@@ -5428,13 +5428,13 @@
         <v>9</v>
       </c>
       <c r="N13" s="31" t="n">
-        <v>93.40000000000001</v>
+        <v>94.5</v>
       </c>
       <c r="O13" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P13" s="31" t="n">
-        <v>83.3</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="Q13" s="31" t="inlineStr">
         <is>
@@ -5453,7 +5453,7 @@
         </is>
       </c>
       <c r="U13" s="31" t="n">
-        <v>81.90000000000001</v>
+        <v>82.3</v>
       </c>
       <c r="V13" s="31" t="inlineStr">
         <is>
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="W13" s="31" t="n">
-        <v>82.59999999999999</v>
+        <v>83</v>
       </c>
       <c r="X13" s="31" t="inlineStr">
         <is>
@@ -5511,7 +5511,7 @@
         </is>
       </c>
       <c r="H14" s="31" t="n">
-        <v>98</v>
+        <v>93.3</v>
       </c>
       <c r="I14" s="31" t="inlineStr">
         <is>
@@ -5519,11 +5519,11 @@
         </is>
       </c>
       <c r="J14" s="31" t="n">
-        <v>85</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="K14" s="31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L14" s="31" t="n">
@@ -5533,17 +5533,17 @@
         <v>9</v>
       </c>
       <c r="N14" s="31" t="n">
-        <v>98.40000000000001</v>
+        <v>82</v>
       </c>
       <c r="O14" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P14" s="31" t="n">
-        <v>90.3</v>
+        <v>82.2</v>
       </c>
       <c r="Q14" s="31" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="R14" s="31" t="n">
@@ -5558,7 +5558,7 @@
         </is>
       </c>
       <c r="U14" s="31" t="n">
-        <v>86.09999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="V14" s="31" t="inlineStr">
         <is>
@@ -5566,7 +5566,7 @@
         </is>
       </c>
       <c r="W14" s="31" t="n">
-        <v>87.2</v>
+        <v>82.3</v>
       </c>
       <c r="X14" s="31" t="inlineStr">
         <is>
@@ -5616,7 +5616,7 @@
         </is>
       </c>
       <c r="H15" s="31" t="n">
-        <v>92.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="I15" s="31" t="inlineStr">
         <is>
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="J15" s="31" t="n">
-        <v>67.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="K15" s="31" t="inlineStr">
         <is>
@@ -5638,13 +5638,13 @@
         <v>9</v>
       </c>
       <c r="N15" s="31" t="n">
-        <v>94.59999999999999</v>
+        <v>95.5</v>
       </c>
       <c r="O15" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P15" s="31" t="n">
-        <v>88.40000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="Q15" s="31" t="inlineStr">
         <is>
@@ -5663,7 +5663,7 @@
         </is>
       </c>
       <c r="U15" s="31" t="n">
-        <v>84.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="V15" s="31" t="inlineStr">
         <is>
@@ -5671,7 +5671,7 @@
         </is>
       </c>
       <c r="W15" s="31" t="n">
-        <v>84.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="X15" s="31" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
         </is>
       </c>
       <c r="J16" s="31" t="n">
-        <v>86.59999999999999</v>
+        <v>86.19999999999999</v>
       </c>
       <c r="K16" s="31" t="inlineStr">
         <is>
@@ -5746,7 +5746,7 @@
         <v>99.5</v>
       </c>
       <c r="O16" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P16" s="31" t="n">
         <v>90.8</v>
@@ -5826,7 +5826,7 @@
         </is>
       </c>
       <c r="H17" s="31" t="n">
-        <v>90.90000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="I17" s="31" t="inlineStr">
         <is>
@@ -5834,7 +5834,7 @@
         </is>
       </c>
       <c r="J17" s="31" t="n">
-        <v>66.59999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="K17" s="31" t="inlineStr">
         <is>
@@ -5848,13 +5848,13 @@
         <v>9</v>
       </c>
       <c r="N17" s="31" t="n">
-        <v>96.8</v>
+        <v>97.3</v>
       </c>
       <c r="O17" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P17" s="31" t="n">
-        <v>85.09999999999999</v>
+        <v>85.3</v>
       </c>
       <c r="Q17" s="31" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
         </is>
       </c>
       <c r="U17" s="31" t="n">
-        <v>83</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="V17" s="31" t="inlineStr">
         <is>
@@ -5881,7 +5881,7 @@
         </is>
       </c>
       <c r="W17" s="31" t="n">
-        <v>83</v>
+        <v>83.2</v>
       </c>
       <c r="X17" s="31" t="inlineStr">
         <is>
@@ -5931,7 +5931,7 @@
         </is>
       </c>
       <c r="H18" s="31" t="n">
-        <v>98</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="I18" s="31" t="inlineStr">
         <is>
@@ -5939,7 +5939,7 @@
         </is>
       </c>
       <c r="J18" s="31" t="n">
-        <v>84.2</v>
+        <v>85.39999999999999</v>
       </c>
       <c r="K18" s="31" t="inlineStr">
         <is>
@@ -5953,13 +5953,13 @@
         <v>9</v>
       </c>
       <c r="N18" s="31" t="n">
-        <v>98.3</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="O18" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P18" s="31" t="n">
-        <v>90.3</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="Q18" s="31" t="inlineStr">
         <is>
@@ -5986,7 +5986,7 @@
         </is>
       </c>
       <c r="W18" s="31" t="n">
-        <v>87.3</v>
+        <v>87.5</v>
       </c>
       <c r="X18" s="31" t="inlineStr">
         <is>
@@ -6036,7 +6036,7 @@
         </is>
       </c>
       <c r="H19" s="31" t="n">
-        <v>97</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="I19" s="31" t="inlineStr">
         <is>
@@ -6044,7 +6044,7 @@
         </is>
       </c>
       <c r="J19" s="31" t="n">
-        <v>67.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="K19" s="31" t="inlineStr">
         <is>
@@ -6058,13 +6058,13 @@
         <v>9</v>
       </c>
       <c r="N19" s="31" t="n">
-        <v>96.40000000000001</v>
+        <v>97</v>
       </c>
       <c r="O19" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P19" s="31" t="n">
-        <v>84.8</v>
+        <v>85</v>
       </c>
       <c r="Q19" s="31" t="inlineStr">
         <is>
@@ -6083,7 +6083,7 @@
         </is>
       </c>
       <c r="U19" s="31" t="n">
-        <v>82.8</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="V19" s="31" t="inlineStr">
         <is>
@@ -6091,7 +6091,7 @@
         </is>
       </c>
       <c r="W19" s="31" t="n">
-        <v>83.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="X19" s="31" t="inlineStr">
         <is>
@@ -6149,11 +6149,11 @@
         </is>
       </c>
       <c r="J20" s="31" t="n">
-        <v>79.2</v>
+        <v>80.8</v>
       </c>
       <c r="K20" s="31" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L20" s="31" t="n">
@@ -6166,7 +6166,7 @@
         <v>96.59999999999999</v>
       </c>
       <c r="O20" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P20" s="31" t="n">
         <v>89</v>
@@ -6254,7 +6254,7 @@
         </is>
       </c>
       <c r="J21" s="31" t="n">
-        <v>83.40000000000001</v>
+        <v>83</v>
       </c>
       <c r="K21" s="31" t="inlineStr">
         <is>
@@ -6268,13 +6268,13 @@
         <v>9</v>
       </c>
       <c r="N21" s="31" t="n">
-        <v>96.8</v>
+        <v>97.3</v>
       </c>
       <c r="O21" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P21" s="31" t="n">
-        <v>89.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="Q21" s="31" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         </is>
       </c>
       <c r="U21" s="31" t="n">
-        <v>85.5</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="V21" s="31" t="inlineStr">
         <is>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="W21" s="31" t="n">
-        <v>86.7</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="X21" s="31" t="inlineStr">
         <is>
@@ -6351,7 +6351,7 @@
         </is>
       </c>
       <c r="H22" s="31" t="n">
-        <v>93.90000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="I22" s="31" t="inlineStr">
         <is>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="J22" s="31" t="n">
-        <v>64.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K22" s="31" t="inlineStr">
         <is>
@@ -6373,13 +6373,13 @@
         <v>9</v>
       </c>
       <c r="N22" s="31" t="n">
-        <v>97.7</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="O22" s="31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P22" s="31" t="n">
-        <v>90</v>
+        <v>90.2</v>
       </c>
       <c r="Q22" s="31" t="inlineStr">
         <is>
@@ -6398,7 +6398,7 @@
         </is>
       </c>
       <c r="U22" s="31" t="n">
-        <v>85.90000000000001</v>
+        <v>86</v>
       </c>
       <c r="V22" s="31" t="inlineStr">
         <is>
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="W22" s="31" t="n">
-        <v>85.59999999999999</v>
+        <v>85.8</v>
       </c>
       <c r="X22" s="31" t="inlineStr">
         <is>
@@ -6475,7 +6475,7 @@
         <v>96.2</v>
       </c>
       <c r="D2" s="31" t="n">
-        <v>85.90000000000001</v>
+        <v>85.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>